<commit_message>
Fix the template's example sheet: it promised rows it never wrote
</commit_message>
<xml_diff>
--- a/data/input_template.xlsx
+++ b/data/input_template.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00;(#,##0.00);-"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,6 +79,11 @@
       <color rgb="001B2438"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="0023272E"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -125,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -170,6 +175,12 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -573,7 +584,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>One row per account for one reporting period. Delete the three example rows below.</t>
+          <t>One row per account for one reporting period. Delete the three example rows below.  * required  † fill either Actual or Budget</t>
         </is>
       </c>
     </row>
@@ -633,12 +644,12 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>Actual *</t>
+          <t>Actual †</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>Budget †</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
@@ -1821,12 +1832,12 @@
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Actual or Budget</t>
         </is>
       </c>
       <c r="C17" s="17" t="inlineStr">
         <is>
-          <t>Actual amount for the reporting period.</t>
+          <t>Actual amount for the reporting period. Fill either this or Budget - a budget-only file is a valid upload, and the app takes one as a second file.</t>
         </is>
       </c>
     </row>
@@ -1836,14 +1847,14 @@
           <t>Budget</t>
         </is>
       </c>
-      <c r="B18" s="21" t="inlineStr">
-        <is>
-          <t>Optional</t>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Actual or Budget</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>Budgeted amount for the same period. Leave the column out if the plan lives in a separate file; you can upload that as a second file.</t>
+          <t>Budgeted amount for the same period. Fill either this or Actual. Leave the column out entirely if the plan lives in a separate file.</t>
         </is>
       </c>
     </row>
@@ -1911,8 +1922,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:AJ18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="17" customWidth="1" min="19" max="19"/>
+    <col width="19" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="11" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
+    <col width="16" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="32" max="32"/>
+    <col width="13" customWidth="1" min="33" max="33"/>
+    <col width="16" customWidth="1" min="34" max="34"/>
+    <col width="15" customWidth="1" min="35" max="35"/>
+    <col width="12" customWidth="1" min="36" max="36"/>
+  </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1927,6 +1976,34 @@
       <c r="F1" s="2" t="n"/>
       <c r="G1" s="2" t="n"/>
       <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="2" t="n"/>
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
+      <c r="S1" s="2" t="n"/>
+      <c r="T1" s="2" t="n"/>
+      <c r="U1" s="2" t="n"/>
+      <c r="V1" s="2" t="n"/>
+      <c r="W1" s="2" t="n"/>
+      <c r="X1" s="2" t="n"/>
+      <c r="Y1" s="2" t="n"/>
+      <c r="Z1" s="2" t="n"/>
+      <c r="AA1" s="2" t="n"/>
+      <c r="AB1" s="2" t="n"/>
+      <c r="AC1" s="2" t="n"/>
+      <c r="AD1" s="2" t="n"/>
+      <c r="AE1" s="2" t="n"/>
+      <c r="AF1" s="2" t="n"/>
+      <c r="AG1" s="2" t="n"/>
+      <c r="AH1" s="2" t="n"/>
+      <c r="AI1" s="2" t="n"/>
+      <c r="AJ1" s="2" t="n"/>
     </row>
     <row r="2" ht="3" customHeight="1">
       <c r="A2" s="4" t="n"/>
@@ -1937,19 +2014,2197 @@
       <c r="F2" s="4" t="n"/>
       <c r="G2" s="4" t="n"/>
       <c r="H2" s="4" t="n"/>
-    </row>
-    <row r="4" ht="52" customHeight="1">
+      <c r="I2" s="4" t="n"/>
+      <c r="J2" s="4" t="n"/>
+      <c r="K2" s="4" t="n"/>
+      <c r="L2" s="4" t="n"/>
+      <c r="M2" s="4" t="n"/>
+      <c r="N2" s="4" t="n"/>
+      <c r="O2" s="4" t="n"/>
+      <c r="P2" s="4" t="n"/>
+      <c r="Q2" s="4" t="n"/>
+      <c r="R2" s="4" t="n"/>
+      <c r="S2" s="4" t="n"/>
+      <c r="T2" s="4" t="n"/>
+      <c r="U2" s="4" t="n"/>
+      <c r="V2" s="4" t="n"/>
+      <c r="W2" s="4" t="n"/>
+      <c r="X2" s="4" t="n"/>
+      <c r="Y2" s="4" t="n"/>
+      <c r="Z2" s="4" t="n"/>
+      <c r="AA2" s="4" t="n"/>
+      <c r="AB2" s="4" t="n"/>
+      <c r="AC2" s="4" t="n"/>
+      <c r="AD2" s="4" t="n"/>
+      <c r="AE2" s="4" t="n"/>
+      <c r="AF2" s="4" t="n"/>
+      <c r="AG2" s="4" t="n"/>
+      <c r="AH2" s="4" t="n"/>
+      <c r="AI2" s="4" t="n"/>
+      <c r="AJ2" s="4" t="n"/>
+    </row>
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>You do not need to trim your export down to the Input sheet. Upload the extract exactly as your system produces it - document numbers, texts, dates, tax codes and any other fields are simply ignored. Flux only needs the account, the amounts and (optionally) department, cost centre and category. The rows below are an illustrative extract.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>doc_no</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>doc_type</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>doc_type_text</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>fiscal_year</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>period</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>period_no</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>doc_date</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>posting_date</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>entry_date</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>entry_time</t>
+        </is>
+      </c>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="L6" s="14" t="inlineStr">
+        <is>
+          <t>header_text</t>
+        </is>
+      </c>
+      <c r="M6" s="14" t="inlineStr">
+        <is>
+          <t>created_by</t>
+        </is>
+      </c>
+      <c r="N6" s="14" t="inlineStr">
+        <is>
+          <t>reversed</t>
+        </is>
+      </c>
+      <c r="O6" s="14" t="inlineStr">
+        <is>
+          <t>entity</t>
+        </is>
+      </c>
+      <c r="P6" s="14" t="inlineStr">
+        <is>
+          <t>company_code</t>
+        </is>
+      </c>
+      <c r="Q6" s="14" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="R6" s="14" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="S6" s="14" t="inlineStr">
+        <is>
+          <t>cost_centre</t>
+        </is>
+      </c>
+      <c r="T6" s="14" t="inlineStr">
+        <is>
+          <t>profit_centre</t>
+        </is>
+      </c>
+      <c r="U6" s="14" t="inlineStr">
+        <is>
+          <t>line_no</t>
+        </is>
+      </c>
+      <c r="V6" s="14" t="inlineStr">
+        <is>
+          <t>account_code</t>
+        </is>
+      </c>
+      <c r="W6" s="14" t="inlineStr">
+        <is>
+          <t>account_name</t>
+        </is>
+      </c>
+      <c r="X6" s="14" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="Y6" s="14" t="inlineStr">
+        <is>
+          <t>expense_type</t>
+        </is>
+      </c>
+      <c r="Z6" s="14" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="AA6" s="14" t="inlineStr">
+        <is>
+          <t>dc_indicator</t>
+        </is>
+      </c>
+      <c r="AB6" s="14" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="AC6" s="14" t="inlineStr">
+        <is>
+          <t>amount_lcy</t>
+        </is>
+      </c>
+      <c r="AD6" s="14" t="inlineStr">
+        <is>
+          <t>fx_rate</t>
+        </is>
+      </c>
+      <c r="AE6" s="14" t="inlineStr">
+        <is>
+          <t>amount_eur</t>
+        </is>
+      </c>
+      <c r="AF6" s="14" t="inlineStr">
+        <is>
+          <t>tax_code</t>
+        </is>
+      </c>
+      <c r="AG6" s="14" t="inlineStr">
+        <is>
+          <t>partner</t>
+        </is>
+      </c>
+      <c r="AH6" s="14" t="inlineStr">
+        <is>
+          <t>assignment</t>
+        </is>
+      </c>
+      <c r="AI6" s="14" t="inlineStr">
+        <is>
+          <t>line_text</t>
+        </is>
+      </c>
+      <c r="AJ6" s="14" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="14" customHeight="1">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>1025000270</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>ZP</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>Payment / bank</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>202506</v>
+      </c>
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="I7" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-03</t>
+        </is>
+      </c>
+      <c r="J7" s="22" t="inlineStr">
+        <is>
+          <t>08:27</t>
+        </is>
+      </c>
+      <c r="K7" s="22" t="inlineStr">
+        <is>
+          <t>Bank-2025-06</t>
+        </is>
+      </c>
+      <c r="L7" s="22" t="inlineStr">
+        <is>
+          <t>Payment / bank 2025-06</t>
+        </is>
+      </c>
+      <c r="M7" s="22" t="inlineStr">
+        <is>
+          <t>BATCHUSER</t>
+        </is>
+      </c>
+      <c r="N7" s="22" t="inlineStr"/>
+      <c r="O7" s="22" t="inlineStr">
+        <is>
+          <t>Flux GmbH</t>
+        </is>
+      </c>
+      <c r="P7" s="22" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="Q7" s="22" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="R7" s="22" t="inlineStr">
+        <is>
+          <t>G&amp;A</t>
+        </is>
+      </c>
+      <c r="S7" s="22" t="inlineStr">
+        <is>
+          <t>GA70300</t>
+        </is>
+      </c>
+      <c r="T7" s="22" t="inlineStr">
+        <is>
+          <t>PC7030</t>
+        </is>
+      </c>
+      <c r="U7" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="V7" s="22" t="inlineStr">
+        <is>
+          <t>7000</t>
+        </is>
+      </c>
+      <c r="W7" s="22" t="inlineStr">
+        <is>
+          <t>Interest expense</t>
+        </is>
+      </c>
+      <c r="X7" s="22" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="Y7" s="22" t="inlineStr">
+        <is>
+          <t>Financing &amp; bank</t>
+        </is>
+      </c>
+      <c r="Z7" s="22" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="AA7" s="22" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AB7" s="22" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC7" s="22" t="n">
+        <v>753.2</v>
+      </c>
+      <c r="AD7" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE7" s="22" t="n">
+        <v>753.2</v>
+      </c>
+      <c r="AF7" s="22" t="inlineStr">
+        <is>
+          <t>**</t>
+        </is>
+      </c>
+      <c r="AG7" s="22" t="inlineStr"/>
+      <c r="AH7" s="22" t="inlineStr">
+        <is>
+          <t>GA70300-202506</t>
+        </is>
+      </c>
+      <c r="AI7" s="22" t="inlineStr">
+        <is>
+          <t>Bank posting 2025-06 - Interest expense</t>
+        </is>
+      </c>
+      <c r="AJ7" s="22" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="14" customHeight="1">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>1025000358</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>PY</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Payroll posting</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>202506</v>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-02</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr">
+        <is>
+          <t>15:03</t>
+        </is>
+      </c>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>Payroll-2025-06</t>
+        </is>
+      </c>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>Payroll posting 2025-06</t>
+        </is>
+      </c>
+      <c r="M8" s="23" t="inlineStr">
+        <is>
+          <t>BATCHUSER</t>
+        </is>
+      </c>
+      <c r="N8" s="23" t="inlineStr"/>
+      <c r="O8" s="23" t="inlineStr">
+        <is>
+          <t>Flux Inc.</t>
+        </is>
+      </c>
+      <c r="P8" s="23" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="Q8" s="23" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="R8" s="23" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="S8" s="23" t="inlineStr">
+        <is>
+          <t>SL20100</t>
+        </is>
+      </c>
+      <c r="T8" s="23" t="inlineStr">
+        <is>
+          <t>PC2010</t>
+        </is>
+      </c>
+      <c r="U8" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="V8" s="23" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="W8" s="23" t="inlineStr">
+        <is>
+          <t>Salaries - Sales</t>
+        </is>
+      </c>
+      <c r="X8" s="23" t="inlineStr">
+        <is>
+          <t>OpEx</t>
+        </is>
+      </c>
+      <c r="Y8" s="23" t="inlineStr">
+        <is>
+          <t>Salaries &amp; wages</t>
+        </is>
+      </c>
+      <c r="Z8" s="23" t="inlineStr">
+        <is>
+          <t>Sales &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AA8" s="23" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AB8" s="23" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AC8" s="23" t="n">
+        <v>16938.93</v>
+      </c>
+      <c r="AD8" s="23" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="AE8" s="23" t="n">
+        <v>15583.81</v>
+      </c>
+      <c r="AF8" s="23" t="inlineStr">
+        <is>
+          <t>**</t>
+        </is>
+      </c>
+      <c r="AG8" s="23" t="inlineStr"/>
+      <c r="AH8" s="23" t="inlineStr">
+        <is>
+          <t>SL20100-202506</t>
+        </is>
+      </c>
+      <c r="AI8" s="23" t="inlineStr">
+        <is>
+          <t>Payroll run 2025-06 - Sales</t>
+        </is>
+      </c>
+      <c r="AJ8" s="23" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="14" customHeight="1">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>1025000369</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>PY</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>Payroll posting</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E9" s="22" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>202506</v>
+      </c>
+      <c r="G9" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="H9" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="I9" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-03</t>
+        </is>
+      </c>
+      <c r="J9" s="22" t="inlineStr">
+        <is>
+          <t>12:23</t>
+        </is>
+      </c>
+      <c r="K9" s="22" t="inlineStr">
+        <is>
+          <t>Payroll-2025-06</t>
+        </is>
+      </c>
+      <c r="L9" s="22" t="inlineStr">
+        <is>
+          <t>Payroll posting 2025-06</t>
+        </is>
+      </c>
+      <c r="M9" s="22" t="inlineStr">
+        <is>
+          <t>BATCHUSER</t>
+        </is>
+      </c>
+      <c r="N9" s="22" t="inlineStr"/>
+      <c r="O9" s="22" t="inlineStr">
+        <is>
+          <t>Flux Inc.</t>
+        </is>
+      </c>
+      <c r="P9" s="22" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="Q9" s="22" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="R9" s="22" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="S9" s="22" t="inlineStr">
+        <is>
+          <t>MK30300</t>
+        </is>
+      </c>
+      <c r="T9" s="22" t="inlineStr">
+        <is>
+          <t>PC3030</t>
+        </is>
+      </c>
+      <c r="U9" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="V9" s="22" t="inlineStr">
+        <is>
+          <t>6010</t>
+        </is>
+      </c>
+      <c r="W9" s="22" t="inlineStr">
+        <is>
+          <t>Salaries - Marketing</t>
+        </is>
+      </c>
+      <c r="X9" s="22" t="inlineStr">
+        <is>
+          <t>OpEx</t>
+        </is>
+      </c>
+      <c r="Y9" s="22" t="inlineStr">
+        <is>
+          <t>Salaries &amp; wages</t>
+        </is>
+      </c>
+      <c r="Z9" s="22" t="inlineStr">
+        <is>
+          <t>Sales &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AA9" s="22" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AB9" s="22" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AC9" s="22" t="n">
+        <v>5818.9</v>
+      </c>
+      <c r="AD9" s="22" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="AE9" s="22" t="n">
+        <v>5353.39</v>
+      </c>
+      <c r="AF9" s="22" t="inlineStr">
+        <is>
+          <t>**</t>
+        </is>
+      </c>
+      <c r="AG9" s="22" t="inlineStr"/>
+      <c r="AH9" s="22" t="inlineStr">
+        <is>
+          <t>MK30300-202506</t>
+        </is>
+      </c>
+      <c r="AI9" s="22" t="inlineStr">
+        <is>
+          <t>Payroll run 2025-06 - Marketing</t>
+        </is>
+      </c>
+      <c r="AJ9" s="22" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="14" customHeight="1">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>1025000379</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>PY</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>Payroll posting</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E10" s="23" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="n">
+        <v>202506</v>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="inlineStr">
+        <is>
+          <t>08:36</t>
+        </is>
+      </c>
+      <c r="K10" s="23" t="inlineStr">
+        <is>
+          <t>Payroll-2025-06</t>
+        </is>
+      </c>
+      <c r="L10" s="23" t="inlineStr">
+        <is>
+          <t>Payroll posting 2025-06</t>
+        </is>
+      </c>
+      <c r="M10" s="23" t="inlineStr">
+        <is>
+          <t>BATCHUSER</t>
+        </is>
+      </c>
+      <c r="N10" s="23" t="inlineStr"/>
+      <c r="O10" s="23" t="inlineStr">
+        <is>
+          <t>Flux Inc.</t>
+        </is>
+      </c>
+      <c r="P10" s="23" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="Q10" s="23" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="R10" s="23" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="S10" s="23" t="inlineStr">
+        <is>
+          <t>EN40300</t>
+        </is>
+      </c>
+      <c r="T10" s="23" t="inlineStr">
+        <is>
+          <t>PC4030</t>
+        </is>
+      </c>
+      <c r="U10" s="23" t="n">
+        <v>17</v>
+      </c>
+      <c r="V10" s="23" t="inlineStr">
+        <is>
+          <t>6001</t>
+        </is>
+      </c>
+      <c r="W10" s="23" t="inlineStr">
+        <is>
+          <t>Payroll taxes &amp; social security</t>
+        </is>
+      </c>
+      <c r="X10" s="23" t="inlineStr">
+        <is>
+          <t>OpEx</t>
+        </is>
+      </c>
+      <c r="Y10" s="23" t="inlineStr">
+        <is>
+          <t>Payroll benefits</t>
+        </is>
+      </c>
+      <c r="Z10" s="23" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="AA10" s="23" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AB10" s="23" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AC10" s="23" t="n">
+        <v>961.77</v>
+      </c>
+      <c r="AD10" s="23" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="AE10" s="23" t="n">
+        <v>884.83</v>
+      </c>
+      <c r="AF10" s="23" t="inlineStr">
+        <is>
+          <t>**</t>
+        </is>
+      </c>
+      <c r="AG10" s="23" t="inlineStr"/>
+      <c r="AH10" s="23" t="inlineStr">
+        <is>
+          <t>EN40300-202506</t>
+        </is>
+      </c>
+      <c r="AI10" s="23" t="inlineStr">
+        <is>
+          <t>Payroll run 2025-06 - Payroll taxes &amp; social security</t>
+        </is>
+      </c>
+      <c r="AJ10" s="23" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="14" customHeight="1">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>1025000858</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>ZP</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>Payment / bank</t>
+        </is>
+      </c>
+      <c r="D11" s="22" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E11" s="22" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>202506</v>
+      </c>
+      <c r="G11" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="H11" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="I11" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-03</t>
+        </is>
+      </c>
+      <c r="J11" s="22" t="inlineStr">
+        <is>
+          <t>08:40</t>
+        </is>
+      </c>
+      <c r="K11" s="22" t="inlineStr">
+        <is>
+          <t>Bank-2025-06</t>
+        </is>
+      </c>
+      <c r="L11" s="22" t="inlineStr">
+        <is>
+          <t>Payment / bank 2025-06</t>
+        </is>
+      </c>
+      <c r="M11" s="22" t="inlineStr">
+        <is>
+          <t>BATCHUSER</t>
+        </is>
+      </c>
+      <c r="N11" s="22" t="inlineStr"/>
+      <c r="O11" s="22" t="inlineStr">
+        <is>
+          <t>Flux Kft.</t>
+        </is>
+      </c>
+      <c r="P11" s="22" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="Q11" s="22" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="R11" s="22" t="inlineStr">
+        <is>
+          <t>G&amp;A</t>
+        </is>
+      </c>
+      <c r="S11" s="22" t="inlineStr">
+        <is>
+          <t>GA70400</t>
+        </is>
+      </c>
+      <c r="T11" s="22" t="inlineStr">
+        <is>
+          <t>PC7040</t>
+        </is>
+      </c>
+      <c r="U11" s="22" t="n">
+        <v>19</v>
+      </c>
+      <c r="V11" s="22" t="inlineStr">
+        <is>
+          <t>7000</t>
+        </is>
+      </c>
+      <c r="W11" s="22" t="inlineStr">
+        <is>
+          <t>Interest expense</t>
+        </is>
+      </c>
+      <c r="X11" s="22" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="Y11" s="22" t="inlineStr">
+        <is>
+          <t>Financing &amp; bank</t>
+        </is>
+      </c>
+      <c r="Z11" s="22" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="AA11" s="22" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AB11" s="22" t="inlineStr">
+        <is>
+          <t>HUF</t>
+        </is>
+      </c>
+      <c r="AC11" s="22" t="n">
+        <v>317760</v>
+      </c>
+      <c r="AD11" s="22" t="n">
+        <v>0.00256</v>
+      </c>
+      <c r="AE11" s="22" t="n">
+        <v>813.46</v>
+      </c>
+      <c r="AF11" s="22" t="inlineStr">
+        <is>
+          <t>**</t>
+        </is>
+      </c>
+      <c r="AG11" s="22" t="inlineStr"/>
+      <c r="AH11" s="22" t="inlineStr">
+        <is>
+          <t>GA70400-202506</t>
+        </is>
+      </c>
+      <c r="AI11" s="22" t="inlineStr">
+        <is>
+          <t>Bank posting 2025-06 - Interest expense</t>
+        </is>
+      </c>
+      <c r="AJ11" s="22" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="14" customHeight="1">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>1025000866</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>ZP</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>Payment / bank</t>
+        </is>
+      </c>
+      <c r="D12" s="23" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E12" s="23" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="F12" s="23" t="n">
+        <v>202506</v>
+      </c>
+      <c r="G12" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-02</t>
+        </is>
+      </c>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-03</t>
+        </is>
+      </c>
+      <c r="J12" s="23" t="inlineStr">
+        <is>
+          <t>18:43</t>
+        </is>
+      </c>
+      <c r="K12" s="23" t="inlineStr">
+        <is>
+          <t>Bank-2025-06</t>
+        </is>
+      </c>
+      <c r="L12" s="23" t="inlineStr">
+        <is>
+          <t>Payment / bank 2025-06</t>
+        </is>
+      </c>
+      <c r="M12" s="23" t="inlineStr">
+        <is>
+          <t>BATCHUSER</t>
+        </is>
+      </c>
+      <c r="N12" s="23" t="inlineStr"/>
+      <c r="O12" s="23" t="inlineStr">
+        <is>
+          <t>Flux Kft.</t>
+        </is>
+      </c>
+      <c r="P12" s="23" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="Q12" s="23" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="R12" s="23" t="inlineStr">
+        <is>
+          <t>G&amp;A</t>
+        </is>
+      </c>
+      <c r="S12" s="23" t="inlineStr">
+        <is>
+          <t>GA70100</t>
+        </is>
+      </c>
+      <c r="T12" s="23" t="inlineStr">
+        <is>
+          <t>PC7010</t>
+        </is>
+      </c>
+      <c r="U12" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="V12" s="23" t="inlineStr">
+        <is>
+          <t>7200</t>
+        </is>
+      </c>
+      <c r="W12" s="23" t="inlineStr">
+        <is>
+          <t>Bank charges</t>
+        </is>
+      </c>
+      <c r="X12" s="23" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="Y12" s="23" t="inlineStr">
+        <is>
+          <t>Financing &amp; bank</t>
+        </is>
+      </c>
+      <c r="Z12" s="23" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="AA12" s="23" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AB12" s="23" t="inlineStr">
+        <is>
+          <t>HUF</t>
+        </is>
+      </c>
+      <c r="AC12" s="23" t="n">
+        <v>73458</v>
+      </c>
+      <c r="AD12" s="23" t="n">
+        <v>0.00256</v>
+      </c>
+      <c r="AE12" s="23" t="n">
+        <v>188.05</v>
+      </c>
+      <c r="AF12" s="23" t="inlineStr">
+        <is>
+          <t>**</t>
+        </is>
+      </c>
+      <c r="AG12" s="23" t="inlineStr"/>
+      <c r="AH12" s="23" t="inlineStr">
+        <is>
+          <t>GA70100-202506</t>
+        </is>
+      </c>
+      <c r="AI12" s="23" t="inlineStr">
+        <is>
+          <t>Bank posting 2025-06 - Bank charges</t>
+        </is>
+      </c>
+      <c r="AJ12" s="23" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="14" customHeight="1">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>1925000010</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>RV</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>Billing document</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="F13" s="22" t="n">
+        <v>202506</v>
+      </c>
+      <c r="G13" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="H13" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-02</t>
+        </is>
+      </c>
+      <c r="I13" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-02</t>
+        </is>
+      </c>
+      <c r="J13" s="22" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="K13" s="22" t="inlineStr">
+        <is>
+          <t>INV-338108</t>
+        </is>
+      </c>
+      <c r="L13" s="22" t="inlineStr">
+        <is>
+          <t>Billing document 2025-06</t>
+        </is>
+      </c>
+      <c r="M13" s="22" t="inlineStr">
+        <is>
+          <t>A.NOVAK</t>
+        </is>
+      </c>
+      <c r="N13" s="22" t="inlineStr"/>
+      <c r="O13" s="22" t="inlineStr">
+        <is>
+          <t>Flux GmbH</t>
+        </is>
+      </c>
+      <c r="P13" s="22" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="Q13" s="22" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="R13" s="22" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="S13" s="22" t="inlineStr">
+        <is>
+          <t>CM10100</t>
+        </is>
+      </c>
+      <c r="T13" s="22" t="inlineStr">
+        <is>
+          <t>PC1010</t>
+        </is>
+      </c>
+      <c r="U13" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="V13" s="22" t="inlineStr">
+        <is>
+          <t>4200</t>
+        </is>
+      </c>
+      <c r="W13" s="22" t="inlineStr">
+        <is>
+          <t>Service revenue - implementation</t>
+        </is>
+      </c>
+      <c r="X13" s="22" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="Y13" s="22" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="Z13" s="22" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="AA13" s="22" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="AB13" s="22" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC13" s="22" t="n">
+        <v>25800.5</v>
+      </c>
+      <c r="AD13" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE13" s="22" t="n">
+        <v>25800.5</v>
+      </c>
+      <c r="AF13" s="22" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="AG13" s="22" t="inlineStr">
+        <is>
+          <t>Vantage Retail Group</t>
+        </is>
+      </c>
+      <c r="AH13" s="22" t="inlineStr">
+        <is>
+          <t>CM10100-202506</t>
+        </is>
+      </c>
+      <c r="AI13" s="22" t="inlineStr">
+        <is>
+          <t>Invoice Vantage Retail Group - Service revenue 2025-06</t>
+        </is>
+      </c>
+      <c r="AJ13" s="22" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="14" customHeight="1">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>1925000018</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>Vendor invoice</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E14" s="23" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="n">
+        <v>202506</v>
+      </c>
+      <c r="G14" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="J14" s="23" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="K14" s="23" t="inlineStr">
+        <is>
+          <t>INV-512123</t>
+        </is>
+      </c>
+      <c r="L14" s="23" t="inlineStr">
+        <is>
+          <t>Vendor invoice 2025-06</t>
+        </is>
+      </c>
+      <c r="M14" s="23" t="inlineStr">
+        <is>
+          <t>S.OKONKWO</t>
+        </is>
+      </c>
+      <c r="N14" s="23" t="inlineStr"/>
+      <c r="O14" s="23" t="inlineStr">
+        <is>
+          <t>Flux GmbH</t>
+        </is>
+      </c>
+      <c r="P14" s="23" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="Q14" s="23" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="R14" s="23" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="S14" s="23" t="inlineStr">
+        <is>
+          <t>OP60300</t>
+        </is>
+      </c>
+      <c r="T14" s="23" t="inlineStr">
+        <is>
+          <t>PC6030</t>
+        </is>
+      </c>
+      <c r="U14" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="V14" s="23" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="W14" s="23" t="inlineStr">
+        <is>
+          <t>Direct materials</t>
+        </is>
+      </c>
+      <c r="X14" s="23" t="inlineStr">
+        <is>
+          <t>COGS</t>
+        </is>
+      </c>
+      <c r="Y14" s="23" t="inlineStr">
+        <is>
+          <t>Materials &amp; components</t>
+        </is>
+      </c>
+      <c r="Z14" s="23" t="inlineStr">
+        <is>
+          <t>Cost of sales</t>
+        </is>
+      </c>
+      <c r="AA14" s="23" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AB14" s="23" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC14" s="23" t="n">
+        <v>11481.55</v>
+      </c>
+      <c r="AD14" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE14" s="23" t="n">
+        <v>11481.55</v>
+      </c>
+      <c r="AF14" s="23" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="AG14" s="23" t="inlineStr">
+        <is>
+          <t>Sentinel Insurance plc</t>
+        </is>
+      </c>
+      <c r="AH14" s="23" t="inlineStr">
+        <is>
+          <t>OP60300-202506</t>
+        </is>
+      </c>
+      <c r="AI14" s="23" t="inlineStr">
+        <is>
+          <t>Sentinel Insurance plc - Direct materials</t>
+        </is>
+      </c>
+      <c r="AJ14" s="23" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="14" customHeight="1">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>1925000310</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>Vendor invoice</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="n">
+        <v>202506</v>
+      </c>
+      <c r="G15" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="H15" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="I15" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="J15" s="22" t="inlineStr">
+        <is>
+          <t>19:19</t>
+        </is>
+      </c>
+      <c r="K15" s="22" t="inlineStr">
+        <is>
+          <t>INV-375552</t>
+        </is>
+      </c>
+      <c r="L15" s="22" t="inlineStr">
+        <is>
+          <t>Vendor invoice 2025-06</t>
+        </is>
+      </c>
+      <c r="M15" s="22" t="inlineStr">
+        <is>
+          <t>J.MEYER</t>
+        </is>
+      </c>
+      <c r="N15" s="22" t="inlineStr"/>
+      <c r="O15" s="22" t="inlineStr">
+        <is>
+          <t>Flux Inc.</t>
+        </is>
+      </c>
+      <c r="P15" s="22" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="Q15" s="22" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="R15" s="22" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="S15" s="22" t="inlineStr">
+        <is>
+          <t>OP60300</t>
+        </is>
+      </c>
+      <c r="T15" s="22" t="inlineStr">
+        <is>
+          <t>PC6030</t>
+        </is>
+      </c>
+      <c r="U15" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="V15" s="22" t="inlineStr">
+        <is>
+          <t>5010</t>
+        </is>
+      </c>
+      <c r="W15" s="22" t="inlineStr">
+        <is>
+          <t>Component costs</t>
+        </is>
+      </c>
+      <c r="X15" s="22" t="inlineStr">
+        <is>
+          <t>COGS</t>
+        </is>
+      </c>
+      <c r="Y15" s="22" t="inlineStr">
+        <is>
+          <t>Materials &amp; components</t>
+        </is>
+      </c>
+      <c r="Z15" s="22" t="inlineStr">
+        <is>
+          <t>Cost of sales</t>
+        </is>
+      </c>
+      <c r="AA15" s="22" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AB15" s="22" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AC15" s="22" t="n">
+        <v>5068.17</v>
+      </c>
+      <c r="AD15" s="22" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="AE15" s="22" t="n">
+        <v>4662.72</v>
+      </c>
+      <c r="AF15" s="22" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="AG15" s="22" t="inlineStr">
+        <is>
+          <t>Delta Components GmbH</t>
+        </is>
+      </c>
+      <c r="AH15" s="22" t="inlineStr">
+        <is>
+          <t>OP60300-202506</t>
+        </is>
+      </c>
+      <c r="AI15" s="22" t="inlineStr">
+        <is>
+          <t>Delta Components GmbH - Component costs</t>
+        </is>
+      </c>
+      <c r="AJ15" s="22" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="14" customHeight="1">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>1925000346</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>Vendor invoice</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E16" s="23" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="F16" s="23" t="n">
+        <v>202506</v>
+      </c>
+      <c r="G16" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="H16" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="I16" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-02</t>
+        </is>
+      </c>
+      <c r="J16" s="23" t="inlineStr">
+        <is>
+          <t>09:32</t>
+        </is>
+      </c>
+      <c r="K16" s="23" t="inlineStr">
+        <is>
+          <t>INV-341124</t>
+        </is>
+      </c>
+      <c r="L16" s="23" t="inlineStr">
+        <is>
+          <t>Vendor invoice 2025-06</t>
+        </is>
+      </c>
+      <c r="M16" s="23" t="inlineStr">
+        <is>
+          <t>J.MEYER</t>
+        </is>
+      </c>
+      <c r="N16" s="23" t="inlineStr"/>
+      <c r="O16" s="23" t="inlineStr">
+        <is>
+          <t>Flux Inc.</t>
+        </is>
+      </c>
+      <c r="P16" s="23" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="Q16" s="23" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="R16" s="23" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="S16" s="23" t="inlineStr">
+        <is>
+          <t>OP60200</t>
+        </is>
+      </c>
+      <c r="T16" s="23" t="inlineStr">
+        <is>
+          <t>PC6020</t>
+        </is>
+      </c>
+      <c r="U16" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="V16" s="23" t="inlineStr">
+        <is>
+          <t>5300</t>
+        </is>
+      </c>
+      <c r="W16" s="23" t="inlineStr">
+        <is>
+          <t>Shipping &amp; fulfilment</t>
+        </is>
+      </c>
+      <c r="X16" s="23" t="inlineStr">
+        <is>
+          <t>COGS</t>
+        </is>
+      </c>
+      <c r="Y16" s="23" t="inlineStr">
+        <is>
+          <t>Logistics &amp; fees</t>
+        </is>
+      </c>
+      <c r="Z16" s="23" t="inlineStr">
+        <is>
+          <t>Cost of sales</t>
+        </is>
+      </c>
+      <c r="AA16" s="23" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AB16" s="23" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AC16" s="23" t="n">
+        <v>4721.03</v>
+      </c>
+      <c r="AD16" s="23" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="AE16" s="23" t="n">
+        <v>4343.35</v>
+      </c>
+      <c r="AF16" s="23" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="AG16" s="23" t="inlineStr">
+        <is>
+          <t>Kovacs Logistics Kft.</t>
+        </is>
+      </c>
+      <c r="AH16" s="23" t="inlineStr">
+        <is>
+          <t>OP60200-202506</t>
+        </is>
+      </c>
+      <c r="AI16" s="23" t="inlineStr">
+        <is>
+          <t>Kovacs Logistics Kft. - Shipping &amp; fulfilment</t>
+        </is>
+      </c>
+      <c r="AJ16" s="23" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="14" customHeight="1">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>1925000583</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>RV</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="inlineStr">
+        <is>
+          <t>Billing document</t>
+        </is>
+      </c>
+      <c r="D17" s="22" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E17" s="22" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="F17" s="22" t="n">
+        <v>202506</v>
+      </c>
+      <c r="G17" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="H17" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-03</t>
+        </is>
+      </c>
+      <c r="I17" s="22" t="inlineStr">
+        <is>
+          <t>2025-06-03</t>
+        </is>
+      </c>
+      <c r="J17" s="22" t="inlineStr">
+        <is>
+          <t>06:34</t>
+        </is>
+      </c>
+      <c r="K17" s="22" t="inlineStr">
+        <is>
+          <t>INV-302922</t>
+        </is>
+      </c>
+      <c r="L17" s="22" t="inlineStr">
+        <is>
+          <t>Billing document 2025-06</t>
+        </is>
+      </c>
+      <c r="M17" s="22" t="inlineStr">
+        <is>
+          <t>S.OKONKWO</t>
+        </is>
+      </c>
+      <c r="N17" s="22" t="inlineStr"/>
+      <c r="O17" s="22" t="inlineStr">
+        <is>
+          <t>Flux Kft.</t>
+        </is>
+      </c>
+      <c r="P17" s="22" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="Q17" s="22" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="R17" s="22" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="S17" s="22" t="inlineStr">
+        <is>
+          <t>CM10100</t>
+        </is>
+      </c>
+      <c r="T17" s="22" t="inlineStr">
+        <is>
+          <t>PC1010</t>
+        </is>
+      </c>
+      <c r="U17" s="22" t="n">
+        <v>17</v>
+      </c>
+      <c r="V17" s="22" t="inlineStr">
+        <is>
+          <t>4200</t>
+        </is>
+      </c>
+      <c r="W17" s="22" t="inlineStr">
+        <is>
+          <t>Service revenue - implementation</t>
+        </is>
+      </c>
+      <c r="X17" s="22" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="Y17" s="22" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="Z17" s="22" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="AA17" s="22" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="AB17" s="22" t="inlineStr">
+        <is>
+          <t>HUF</t>
+        </is>
+      </c>
+      <c r="AC17" s="22" t="n">
+        <v>5367385</v>
+      </c>
+      <c r="AD17" s="22" t="n">
+        <v>0.00256</v>
+      </c>
+      <c r="AE17" s="22" t="n">
+        <v>13740.51</v>
+      </c>
+      <c r="AF17" s="22" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="AG17" s="22" t="inlineStr">
+        <is>
+          <t>Vantage Retail Group</t>
+        </is>
+      </c>
+      <c r="AH17" s="22" t="inlineStr">
+        <is>
+          <t>CM10100-202506</t>
+        </is>
+      </c>
+      <c r="AI17" s="22" t="inlineStr">
+        <is>
+          <t>Invoice Vantage Retail Group - Service revenue 2025-06</t>
+        </is>
+      </c>
+      <c r="AJ17" s="22" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="14" customHeight="1">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>1925000586</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>RV</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>Billing document</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="F18" s="23" t="n">
+        <v>202506</v>
+      </c>
+      <c r="G18" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-03</t>
+        </is>
+      </c>
+      <c r="I18" s="23" t="inlineStr">
+        <is>
+          <t>2025-06-05</t>
+        </is>
+      </c>
+      <c r="J18" s="23" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="K18" s="23" t="inlineStr">
+        <is>
+          <t>INV-830665</t>
+        </is>
+      </c>
+      <c r="L18" s="23" t="inlineStr">
+        <is>
+          <t>Billing document 2025-06</t>
+        </is>
+      </c>
+      <c r="M18" s="23" t="inlineStr">
+        <is>
+          <t>J.MEYER</t>
+        </is>
+      </c>
+      <c r="N18" s="23" t="inlineStr"/>
+      <c r="O18" s="23" t="inlineStr">
+        <is>
+          <t>Flux Kft.</t>
+        </is>
+      </c>
+      <c r="P18" s="23" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="Q18" s="23" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="R18" s="23" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="S18" s="23" t="inlineStr">
+        <is>
+          <t>CM10100</t>
+        </is>
+      </c>
+      <c r="T18" s="23" t="inlineStr">
+        <is>
+          <t>PC1010</t>
+        </is>
+      </c>
+      <c r="U18" s="23" t="n">
+        <v>17</v>
+      </c>
+      <c r="V18" s="23" t="inlineStr">
+        <is>
+          <t>4210</t>
+        </is>
+      </c>
+      <c r="W18" s="23" t="inlineStr">
+        <is>
+          <t>Support contract revenue</t>
+        </is>
+      </c>
+      <c r="X18" s="23" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="Y18" s="23" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="Z18" s="23" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="AA18" s="23" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="AB18" s="23" t="inlineStr">
+        <is>
+          <t>HUF</t>
+        </is>
+      </c>
+      <c r="AC18" s="23" t="n">
+        <v>8563651</v>
+      </c>
+      <c r="AD18" s="23" t="n">
+        <v>0.00256</v>
+      </c>
+      <c r="AE18" s="23" t="n">
+        <v>21922.95</v>
+      </c>
+      <c r="AF18" s="23" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="AG18" s="23" t="inlineStr">
+        <is>
+          <t>Vantage Retail Group</t>
+        </is>
+      </c>
+      <c r="AH18" s="23" t="inlineStr">
+        <is>
+          <t>CM10100-202506</t>
+        </is>
+      </c>
+      <c r="AI18" s="23" t="inlineStr">
+        <is>
+          <t>Invoice Vantage Retail Group - Support contract revenue 2025-06</t>
+        </is>
+      </c>
+      <c r="AJ18" s="23" t="inlineStr">
+        <is>
+          <t>AR</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A4:AJ4"/>
+    <mergeCell ref="A2:AJ2"/>
+    <mergeCell ref="A1:AJ1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Stop the template's example sheet from outscoring its own Input sheet
</commit_message>
<xml_diff>
--- a/data/input_template.xlsx
+++ b/data/input_template.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to fill" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example - full GL export" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to fill" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example - full GL export" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1612,9 +1613,12 @@
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A3:K3"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="D6:D68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose Revenue, COGS, OpEx or Other (or leave blank)." prompt="Optional - leave blank and Flux infers it from the account code." type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="D6:D68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose Revenue, COGS, OpEx or Other (or leave blank)." prompt="Optional - leave blank and Flux works it out from the code and the name." type="list">
       <formula1>"Revenue,COGS,OpEx,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E6:E68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Not one of the standard types - your own names are fine too." prompt="Pick one, or type your own name." type="list" errorStyle="warning">
+      <formula1>Lists!$A$2:$A$18</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1622,6 +1626,149 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Expense types - the list behind the dropdown on Input.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Salaries &amp; wages</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Payroll benefits</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Employee incentives</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>External staff / contractors</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Marketing &amp; advertising</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>External professional fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IT &amp; software</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Facilities &amp; office</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Travel &amp; entertainment</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Materials &amp; components</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Direct labour</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Hosting &amp; infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Third-party licences</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Logistics &amp; fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; amortisation</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Financing &amp; bank</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001B2438"/>
@@ -1653,14 +1800,14 @@
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>This template is optional</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="52" customHeight="1">
+          <t>Why this template is the recommended way in</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="88" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>Flux reads most general-ledger and trial-balance exports as they are: it recognises common column names in English and Hungarian, matches close variants, and infers fields from the data. Use this template only if your export does not map cleanly, or if you are building the file by hand.</t>
+          <t>Flux also reads general-ledger and trial-balance exports as they are - it recognises column names in English, Hungarian and German, classifies the accounts from their codes and names, and drops the subtotal rows a printed report carries. The numbers come out the same either way when it reads the file correctly. What this template removes is the reading: nothing to map, no chart of accounts to recognise, no expense types inferred from account names, and no printed totals to filter out. Use it when the pack has to be right the first time; upload your raw export when you would rather check four assumptions than fill a sheet.</t>
         </is>
       </c>
     </row>
@@ -1752,7 +1899,7 @@
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>Revenue / COGS / OpEx / Other. Left blank, Flux infers it from the account code.</t>
+          <t>Revenue / COGS / OpEx / Other. Left blank, Flux works it out from the account code and the account name together, and reports what it assumed.</t>
         </is>
       </c>
     </row>
@@ -1769,7 +1916,7 @@
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>Natural classification, e.g. Salaries &amp; wages, Marketing, External professional fees. Drives the Expense Report sheet.</t>
+          <t>Natural classification - pick from the dropdown, or use your own names. Drives the Expense Report sheet. Left blank, Flux infers it from the account name, which is the weakest guess it makes.</t>
         </is>
       </c>
     </row>
@@ -1899,7 +2046,7 @@
     <row r="25" ht="52" customHeight="1">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>Amounts can use either European (1.234.567,89) or US (1,234,567.89) formatting; Flux parses both. Enter positive magnitudes: revenue as a positive number and costs as positive numbers too. Fill one period per file, and set the reporting period in the app sidebar.</t>
+          <t>Amounts can use either European (1.234.567,89) or US (1,234,567.89) formatting; Flux parses both. Enter positive magnitudes: revenue as a positive number and costs as positive numbers too. Several periods in one file are fine and are what produce the year-to-date columns - fill the Accounting period column and Flux reports the latest month that carries postings. With no period column at all, the app asks what to label the report.</t>
         </is>
       </c>
     </row>
@@ -1915,7 +2062,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001B2438"/>

</xml_diff>

<commit_message>
Size every block on the template from its own text
</commit_message>
<xml_diff>
--- a/data/input_template.xlsx
+++ b/data/input_template.xlsx
@@ -1779,7 +1779,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="74" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -1804,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="88" customHeight="1">
+    <row r="5" ht="100" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Flux also reads general-ledger and trial-balance exports as they are - it recognises column names in English, Hungarian and German, classifies the accounts from their codes and names, and drops the subtotal rows a printed report carries. The numbers come out the same either way when it reads the file correctly. What this template removes is the reading: nothing to map, no chart of accounts to recognise, no expense types inferred from account names, and no printed totals to filter out. Use it when the pack has to be right the first time; upload your raw export when you would rather check four assumptions than fill a sheet.</t>
@@ -1835,7 +1835,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="40" customHeight="1">
       <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Accounting period</t>
@@ -1886,7 +1886,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="40" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Category</t>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
+    <row r="13" ht="55" customHeight="1">
       <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Expense type</t>
@@ -1920,7 +1920,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="14" ht="40" customHeight="1">
       <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Entity</t>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
+    <row r="16" ht="55" customHeight="1">
       <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Cost centre</t>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="55" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Actual</t>
@@ -1988,7 +1988,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
+    <row r="18" ht="40" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Budget</t>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="96" customHeight="1">
+    <row r="22" ht="160" customHeight="1">
       <c r="A22" s="13" t="inlineStr">
         <is>
           <t>Cost centres sit inside departments; the department is the roll-up level. Put the department in one column and the cost centre it belongs to in the next, on the same row - for example Engineering / QA &amp; Release, or Marketing / MK30200. Enter the cost centre in your own coding scheme - CC1200, EN40300 and 4100-02 are all fine, Flux takes it as it is. Post revenue the way your own system does: many companies book revenue to a commercial or sales cost centre (and credit notes always follow the cost centre of the original entry), while others track revenue by profit centre only. Flux accepts either - fill the columns if you have them, leave them blank if you do not. Every optional dimension you fill adds a sheet to the pack: expense type gives the Expense Report, department and cost centre give the Departments &amp; Cost Centres view, and more than one entity gives a consolidation sheet. Without them you still get the P&amp;L and the account-level variance. The departmental view reports spend, so revenue rows are excluded from it either way.</t>
@@ -2043,7 +2043,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="52" customHeight="1">
+    <row r="25" ht="85" customHeight="1">
       <c r="A25" s="13" t="inlineStr">
         <is>
           <t>Amounts can use either European (1.234.567,89) or US (1,234,567.89) formatting; Flux parses both. Enter positive magnitudes: revenue as a positive number and costs as positive numbers too. Several periods in one file are fine and are what produce the year-to-date columns - fill the Accounting period column and Flux reports the latest month that carries postings. With no period column at all, the app asks what to label the report.</t>

</xml_diff>

<commit_message>
Say what each template column gives you, not whether it is required
</commit_message>
<xml_diff>
--- a/data/input_template.xlsx
+++ b/data/input_template.xlsx
@@ -585,7 +585,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>One row per account for one reporting period. Delete the three example rows below.  * required  † fill either Actual or Budget</t>
+          <t>One row per account per period. Delete the three example rows below.  * required  † fill one of these two  ·  every other column adds a sheet or a comparison - see How to fill</t>
         </is>
       </c>
     </row>
@@ -1775,11 +1775,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="74" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -1804,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="100" customHeight="1">
+    <row r="5" ht="115" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Flux also reads general-ledger and trial-balance exports as they are - it recognises column names in English, Hungarian and German, classifies the accounts from their codes and names, and drops the subtotal rows a printed report carries. The numbers come out the same either way when it reads the file correctly. What this template removes is the reading: nothing to map, no chart of accounts to recognise, no expense types inferred from account names, and no printed totals to filter out. Use it when the pack has to be right the first time; upload your raw export when you would rather check four assumptions than fill a sheet.</t>
@@ -1818,244 +1818,252 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+    <row r="8" ht="70" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Only the account code, the account name and one amount column are strictly required - that is the whole of what Flux needs to produce a P&amp;L. Everything else turns that into the full pack: each column adds a sheet, a comparison or removes a guess, and the middle column below says which. Fill every one you have and the pack is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>What it gives you</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
+    <row r="11" ht="55" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>Accounting period</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C9" s="17" t="inlineStr">
-        <is>
-          <t>The period the line belongs to, e.g. 2025-06. Fill it if the file covers more than one month; Flux then reports one period at a time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>YTD and run-rate columns</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>The period the line belongs to, e.g. 2025-06. Several periods in one file is what produces the year-to-date view; Flux reports the latest month that carries postings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Account code</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Everything - required</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>Text or number, e.g. 4100.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="15" t="inlineStr">
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Account name</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>Everything - required</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>Free text description.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
+    <row r="14" ht="55" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>Removes a guess</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
         <is>
           <t>Revenue / COGS / OpEx / Other. Left blank, Flux works it out from the account code and the account name together, and reports what it assumed.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="55" customHeight="1">
-      <c r="A13" s="15" t="inlineStr">
+    <row r="15" ht="55" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Expense type</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C13" s="17" t="inlineStr">
-        <is>
-          <t>Natural classification - pick from the dropdown, or use your own names. Drives the Expense Report sheet. Left blank, Flux infers it from the account name, which is the weakest guess it makes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Expense Report sheet</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>Natural classification - pick from the dropdown, or use your own names. Left blank, Flux infers it from the account name, which is the weakest guess it makes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Entity</t>
         </is>
       </c>
-      <c r="B14" s="21" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C14" s="13" t="inlineStr">
-        <is>
-          <t>Legal entity or company code. With more than one, the pack adds a consolidation sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>By Entity sheet</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>Legal entity or company code. The consolidation sheet appears once there is more than one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Departments &amp; CCs sheet</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>The roll-up level, e.g. Engineering.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="55" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
+    <row r="18" ht="55" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Cost centre</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>Cost centres inside it</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
         <is>
           <t>The cost centre inside that department, in your own coding scheme, e.g. CC1200, EN40300 or 4100-02. Must belong to the department in the same row.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="55" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
-        <is>
-          <t>Actual or Budget</t>
-        </is>
-      </c>
-      <c r="C17" s="17" t="inlineStr">
-        <is>
-          <t>Actual amount for the reporting period. Fill either this or Budget - a budget-only file is a valid upload, and the app takes one as a second file.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>Fill one of these two</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>Actual amount for the reporting period. A budget-only file is a valid upload, and the app takes one as a second file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="B18" s="19" t="inlineStr">
-        <is>
-          <t>Actual or Budget</t>
-        </is>
-      </c>
-      <c r="C18" s="13" t="inlineStr">
-        <is>
-          <t>Budgeted amount for the same period. Fill either this or Actual. Leave the column out entirely if the plan lives in a separate file.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>Fill one of these two</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>Budgeted amount for the same period. Leave the column out entirely if the plan lives in a separate file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>Prior year actual</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C19" s="17" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Prior-year comparison</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>The same period last year, actual (not last year's budget).</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="12" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>Department and cost centre</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="160" customHeight="1">
-      <c r="A22" s="13" t="inlineStr">
+    <row r="24" ht="175" customHeight="1">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>Cost centres sit inside departments; the department is the roll-up level. Put the department in one column and the cost centre it belongs to in the next, on the same row - for example Engineering / QA &amp; Release, or Marketing / MK30200. Enter the cost centre in your own coding scheme - CC1200, EN40300 and 4100-02 are all fine, Flux takes it as it is. Post revenue the way your own system does: many companies book revenue to a commercial or sales cost centre (and credit notes always follow the cost centre of the original entry), while others track revenue by profit centre only. Flux accepts either - fill the columns if you have them, leave them blank if you do not. Every optional dimension you fill adds a sheet to the pack: expense type gives the Expense Report, department and cost centre give the Departments &amp; Cost Centres view, and more than one entity gives a consolidation sheet. Without them you still get the P&amp;L and the account-level variance. The departmental view reports spend, so revenue rows are excluded from it either way.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Numbers and periods</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="85" customHeight="1">
-      <c r="A25" s="13" t="inlineStr">
+    <row r="27" ht="85" customHeight="1">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>Amounts can use either European (1.234.567,89) or US (1,234,567.89) formatting; Flux parses both. Enter positive magnitudes: revenue as a positive number and costs as positive numbers too. Several periods in one file are fine and are what produce the year-to-date columns - fill the Accounting period column and Flux reports the latest month that carries postings. With no period column at all, the app asks what to label the report.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A25:C25"/>
+  <mergeCells count="6">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A24:C24"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>